<commit_message>
Prepare journal-neutral v1.3.1 metadata release
</commit_message>
<xml_diff>
--- a/tables/Table_1_cohort_characteristics.xlsx
+++ b/tables/Table_1_cohort_characteristics.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd32786d89a384b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R695c8b324f0c453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0c1b26ace0f5429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R87d9359851a2441e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -371,7 +371,7 @@
         <x:v>Manuscript</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>Scientific_Reports_Manuscript.docx</x:v>
+        <x:v>Legacy manuscript source (journal-specific filename normalized in v1.3.1)</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>